<commit_message>
Model completed, BOM completed
</commit_message>
<xml_diff>
--- a/RotatingDrive/RotatingDrive.xlsx
+++ b/RotatingDrive/RotatingDrive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\NFSROBOT\HALS-Documentation\GitHub-RotatingDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A558E1-59E3-411D-ADBE-4F6E761E2153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424ADF6A-C529-4D1F-962C-F8E5A4B82A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2415" yWindow="4380" windowWidth="23280" windowHeight="11100" activeTab="1" xr2:uid="{3D4F8E6E-17CE-436E-B881-B7A2EBED38DB}"/>
+    <workbookView xWindow="30375" yWindow="1770" windowWidth="19740" windowHeight="11100" activeTab="1" xr2:uid="{3D4F8E6E-17CE-436E-B881-B7A2EBED38DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Rotating-Drive" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="143">
   <si>
     <t>RD020</t>
   </si>
@@ -79,10 +79,6 @@
   </si>
   <si>
     <t>RD009</t>
-  </si>
-  <si>
-    <t>The casing of the drive is also needed for supporting the cable spiral coming from the arm -assy and going into the foot. Checklist C013 
-I added 2 supports  angled 45 degrees from central axis and on one support an endplate to block the cable-chain from moving too much.  So far this works fine.</t>
   </si>
   <si>
     <t>RD008</t>
@@ -101,9 +97,6 @@
     <t>RD006</t>
   </si>
   <si>
-    <t>Another issue is that all the belt lenth calculators i could access on the internet gave wrong results, very curious.  But it means i have to device a calculator in Fusion 360 to satisfy the need. Checklist C004. Stopped, the https://www.dold-mechatronik.de/Zahnriemen  provides a close enough ressult.</t>
-  </si>
-  <si>
     <t>RD005</t>
   </si>
   <si>
@@ -113,9 +106,6 @@
     <t>RD004</t>
   </si>
   <si>
-    <t>So a second proto made and this one did rotate the test arm in a controllable way up to ~1 degree steps.  Use of a reduction gearing of 10:1 plus HTD3M toothed belt and a 270:20 pulley ratio. Thus 135:1. With appropriate GRBL settings for acceleration and speed a 1 degree step is possible and a 180 degree sweep in ~ 9 seconds. Checklist C002, Done.</t>
-  </si>
-  <si>
     <t>RD003</t>
   </si>
   <si>
@@ -293,24 +283,15 @@
     <t>RD-CH001</t>
   </si>
   <si>
-    <t>Specific for the gravity tripod, using 3d Model: TripodCentralMount-Replica</t>
-  </si>
-  <si>
     <t>RD-CH002</t>
   </si>
   <si>
     <t>RD-CH003</t>
   </si>
   <si>
-    <t>Main chassis beam</t>
-  </si>
-  <si>
     <t>CableChain-mount- Chassis-side</t>
   </si>
   <si>
-    <t>specific for the closed belt size HTD3M-1068mm ; 3D printed, using PETG (Rapid PETG)</t>
-  </si>
-  <si>
     <t>3D printed, using PETG (Rapid PETG), glued to chassis beam with cyanoacrylarte (degrease first!)</t>
   </si>
   <si>
@@ -387,9 +368,6 @@
   </si>
   <si>
     <t>Flathead-bolt-M5x15mm (www.systeal.com)</t>
-  </si>
-  <si>
-    <t>For M5 and M8 bolts the holes are tapped , use a bit of isopropyl-alcohol to reduce friction and temperature raising. Practice this before final.</t>
   </si>
   <si>
     <t>The Nema17 motor cable connection requires an endcap to secure the cable mount to the motor.</t>
@@ -452,13 +430,53 @@
   </si>
   <si>
     <t>HTD3M-1068mm Closed belt</t>
+  </si>
+  <si>
+    <t>Another issue is that all the belt lenth calculators i could access on the internet gave wrong results, very curious.  But it means i have to device a calculator in Fusion 360 to satisfy the need. Checklist C004. Stopped, the https://www.dold-mechatronik.de/Zahnriemen  provides a close enough ressult, around 1mm tolerance.</t>
+  </si>
+  <si>
+    <t>So a second proto made and this one did rotate the test arm in a controllable way up to ~1 degree steps.  Use of a reduction gearing of 10:1 plus HTD3M-9mm toothed belt and a 270:20 pulley ratio. Thus 135:1. With appropriate GRBL settings for acceleration and speed a 1 degree step is possible and a 180 degree sweep in ~ 9 seconds. Checklist C002, Done.</t>
+  </si>
+  <si>
+    <t>The casing initially planned of the drive and is also needed for supporting the cable spiral coming from the arm -assy and going into the foot. Checklist C013 . Decided not to make a casing.
+Instead I added 2 rigs  angled 45 degrees from central axis and on one support an endplate to block the cable-chain from moving too much.  So far this works fine.</t>
+  </si>
+  <si>
+    <t>For M5 and M8 bolts the holes are threaded , use a bit of isopropyl-alcohol to reduce friction and temperature raising. Practice this before final.</t>
+  </si>
+  <si>
+    <t>CHASSIS (Main chassis beam)</t>
+  </si>
+  <si>
+    <t>Specific for the gravity tripod, using 3d Model: TripodCentralMount-Replica. HUB glued into the main chassis beam, while being very well aligned. Degrease the surfaces thoroughly!</t>
+  </si>
+  <si>
+    <t>Specific for the closed belt size HTD3M-1068mm ; 3D printed, using PETG (Rapid PETG)</t>
+  </si>
+  <si>
+    <t>Allen bolt M4x15 + washer</t>
+  </si>
+  <si>
+    <t>To mount the motor-reductiongear combo to the Motormount.</t>
+  </si>
+  <si>
+    <t>Countersunk-screw 3.2x10mm</t>
+  </si>
+  <si>
+    <t>RD-MP014</t>
+  </si>
+  <si>
+    <t>RD-MP015</t>
+  </si>
+  <si>
+    <t>To mount the Bottom bearing flancge to the 270t main pulley. Note: with thick leather or similar fibrous material washers in between.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -503,6 +521,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -629,7 +655,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -658,7 +684,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1137,74 +1174,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>20</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1212,14 +1249,14 @@
         <v>13</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="16" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1228,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1236,7 +1273,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -1244,7 +1281,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1260,7 +1297,7 @@
         <v>5</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1268,7 +1305,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1276,7 +1313,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1318,7 +1355,7 @@
     <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1328,709 +1365,733 @@
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="E3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="F3" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="14" t="s">
+    </row>
+    <row r="4" spans="1:6" s="19" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="17">
+        <v>1</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="11">
-        <v>1</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>84</v>
+      <c r="F4" s="18" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="D5" s="11">
         <v>1</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>89</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D6" s="11">
         <v>1</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D7" s="11">
         <v>1</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D8" s="10">
         <v>1</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D9" s="10">
         <v>1</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D10" s="10">
         <v>2</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="10">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>96</v>
-      </c>
-      <c r="D11" s="10">
-        <v>1</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D12" s="10">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D13" s="10">
         <v>1</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D14" s="10">
         <v>1</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D15" s="10">
         <v>2</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D16" s="10">
         <v>1</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>62</v>
-      </c>
       <c r="D17" s="10">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D18" s="10">
         <v>1</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B19" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>69</v>
-      </c>
       <c r="D19" s="10">
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D20" s="10">
         <v>4</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B21" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="10">
+        <v>1</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="12" t="s">
         <v>73</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="10">
-        <v>1</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="D22" s="10">
         <v>3</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D23" s="10">
         <v>2</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D24" s="10">
         <v>1</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D25" s="10">
         <v>1</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D26" s="10">
         <v>1</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D27" s="10">
         <v>2</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>42</v>
+        <v>140</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>49</v>
+        <v>137</v>
       </c>
       <c r="D29" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>44</v>
+        <v>141</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>50</v>
+        <v>139</v>
       </c>
       <c r="D30" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>40</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D31" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F31" s="11"/>
+        <v>36</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D32" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F32" s="11"/>
+        <v>36</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D33" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>54</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F33" s="11"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="11" t="s">
-        <v>48</v>
-      </c>
       <c r="C34" s="11" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D34" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>56</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="F34" s="11"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="D35" s="11">
         <v>2</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>121</v>
+        <v>52</v>
       </c>
       <c r="D36" s="11">
         <v>1</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>122</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="D37" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>124</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
+      <c r="A38" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D38" s="11">
+        <v>1</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
+      <c r="A39" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D39" s="11">
+        <v>1</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="11"/>

</xml_diff>